<commit_message>
Add DRAFT watermark to every tab of the audit workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PVCfJqUd1kQ4cq8YAWYC5E
</commit_message>
<xml_diff>
--- a/codebase-audit-report/codebase-audit-metrics.xlsx
+++ b/codebase-audit-report/codebase-audit-metrics.xlsx
@@ -2720,10 +2720,522 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>101160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>245520</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>110520</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>321480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>809280</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>115560</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>104400</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>41760</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>479880</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2712600</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>130680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2712600</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="9524880"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>93</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2712600</xdr:colOff>
+      <xdr:row>112</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="18097560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>138</xdr:row>
+      <xdr:rowOff>130680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2712600</xdr:colOff>
+      <xdr:row>157</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="26669880"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>183</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2712600</xdr:colOff>
+      <xdr:row>202</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="35242560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>228</xdr:row>
+      <xdr:rowOff>130680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2712600</xdr:colOff>
+      <xdr:row>247</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Image 6" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId6"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="43814880"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1796040</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>493200</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>54360</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="571680"/>
+          <a:ext cx="13334760" cy="18020880"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>53280</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2740,7 +3252,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="23" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2762,10 +3274,47 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>53280</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing17.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2782,7 +3331,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="25" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2804,10 +3353,47 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>53280</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing18.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2824,7 +3410,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="27" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2846,10 +3432,47 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>53280</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing19.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2866,7 +3489,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="29" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2888,10 +3511,89 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>53280</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>456840</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing20.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2908,7 +3610,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="31" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2930,35 +3632,370 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>53280</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1232280</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>321480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>104400</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>130680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>104400</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="9524880"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>268560</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>34200</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>131040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>739080</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>130680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>739080</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>140040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="9524880"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>321480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2430720</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>27720</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2967,18 +4004,18 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>131040</xdr:rowOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>321480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>493200</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>54360</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>104400</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>230400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2987,8 +4024,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="571680"/>
-          <a:ext cx="13334760" cy="18020880"/>
+          <a:off x="0" y="952560"/>
+          <a:ext cx="4333680" cy="3628800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3316,6 +4353,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3715,6 +4753,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4135,6 +5174,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4231,6 +5271,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9860,6 +10901,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10664,6 +11706,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>